<commit_message>
Clarify FY2026 audit scope
</commit_message>
<xml_diff>
--- a/outputs/fy2026_prediction_validation.xlsx
+++ b/outputs/fy2026_prediction_validation.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FY2026 Actuals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Raw" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Note" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FY2026 Actuals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Raw" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,6 +440,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Post-model forecast audit only</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Model base year remains</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Writes to model inputs</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Used for assumption tuning</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -856,7 +935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1486,7 +1565,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>